<commit_message>
Refactor UAT checklist reduction logic in reduce_test_plans.py to enforce hard coverage constraints and improve scoring methodology
- Updated reduction algorithm to deterministically reduce UAT checklists while preserving at least one checklist check per AC Ref and core case type.
- Introduced scoring system based on priority, fidelity, evidence availability, and case type to determine which checks to drop.
- Enhanced KPI reporting to include detailed metrics on AC coverage and priority reliability before and after reduction.
- Modified output summary format to provide clearer insights into dropped checks and their associated sections.
- Updated multiple Excel files in the reduced test plans directory to reflect changes in the reduction process.
</commit_message>
<xml_diff>
--- a/uat-test-plans-reduced30/G2-16011-view-of-the-customer-customer-information.xlsx
+++ b/uat-test-plans-reduced30/G2-16011-view-of-the-customer-customer-information.xlsx
@@ -597,7 +597,7 @@
       </c>
       <c r="B12" s="3" t="inlineStr">
         <is>
-          <t>[Reduced ~25% — 6/8 checks retained, lowest-priority sections dropped] 1 UI story (G2-20728) mapped to 8 business checks and 5 AC coverage rows. 1 evaluation spike (G2-25652) excluded from executable UAT scope.</t>
+          <t>[Reduced V2 ~25% — 6/8 checks retained; AC and core-case coverage guardrails enforced] 1 UI story (G2-20728) mapped to 8 business checks and 5 AC coverage rows. 1 evaluation spike (G2-25652) excluded from executable UAT scope.</t>
         </is>
       </c>
     </row>
@@ -669,7 +669,7 @@
       </c>
       <c r="B18" s="3" t="inlineStr">
         <is>
-          <t>payload_bytes=7545; payload_chars=7531; est_tokens~1883; checklist_rows=6; matrix_rows=4; exploratory_rows=2</t>
+          <t>payload_bytes=7993; payload_chars=7979; est_tokens~1995; checklist_rows=6; matrix_rows=5; exploratory_rows=2</t>
         </is>
       </c>
     </row>
@@ -701,7 +701,7 @@
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
     <col width="37" customWidth="1" min="2" max="2"/>
-    <col width="19" customWidth="1" min="3" max="3"/>
+    <col width="21" customWidth="1" min="3" max="3"/>
     <col width="50" customWidth="1" min="4" max="4"/>
     <col width="50" customWidth="1" min="5" max="5"/>
     <col width="50" customWidth="1" min="6" max="6"/>
@@ -892,10 +892,10 @@
       <c r="G5" s="5" t="inlineStr"/>
       <c r="H5" s="5" t="inlineStr"/>
     </row>
-    <row r="6" ht="64" customHeight="1">
+    <row r="6" ht="49" customHeight="1">
       <c r="A6" s="5" t="inlineStr">
         <is>
-          <t>UAT-005</t>
+          <t>UAT-006</t>
         </is>
       </c>
       <c r="B6" s="5" t="inlineStr">
@@ -905,32 +905,32 @@
       </c>
       <c r="C6" s="5" t="inlineStr">
         <is>
-          <t>Access &amp; Roles</t>
+          <t>Copy Behavior</t>
         </is>
       </c>
       <c r="D6" s="5" t="inlineStr">
         <is>
-          <t>No unintended masking of parentUrn for business users</t>
+          <t>User can copy parentUrn from the customer profile</t>
         </is>
       </c>
       <c r="E6" s="5" t="inlineStr">
         <is>
-          <t>Repeat profile access with another business user role responsible for reservation creation and verify parentUrn is shown in the same area.</t>
+          <t>Select and copy the displayed parentUrn value using keyboard or UI copy interaction if available.</t>
         </is>
       </c>
       <c r="F6" s="5" t="inlineStr">
         <is>
-          <t>The field is consistently visible across intended reservation-related roles.
-Field placement and readability are consistent.</t>
+          <t>Copy action succeeds without errors.
+Clipboard contains a value matching the displayed parentUrn.</t>
         </is>
       </c>
       <c r="G6" s="5" t="inlineStr"/>
       <c r="H6" s="5" t="inlineStr"/>
     </row>
-    <row r="7" ht="49" customHeight="1">
+    <row r="7" ht="64" customHeight="1">
       <c r="A7" s="5" t="inlineStr">
         <is>
-          <t>UAT-006</t>
+          <t>UAT-007</t>
         </is>
       </c>
       <c r="B7" s="5" t="inlineStr">
@@ -940,23 +940,23 @@
       </c>
       <c r="C7" s="5" t="inlineStr">
         <is>
-          <t>Copy Behavior</t>
+          <t>Concierge Handover</t>
         </is>
       </c>
       <c r="D7" s="5" t="inlineStr">
         <is>
-          <t>User can copy parentUrn from the customer profile</t>
+          <t>Copied parentUrn pastes into Concierge input without format problems</t>
         </is>
       </c>
       <c r="E7" s="5" t="inlineStr">
         <is>
-          <t>Select and copy the displayed parentUrn value using keyboard or UI copy interaction if available.</t>
+          <t>Paste the copied parentUrn into the target Concierge field used during reservation creation and review the pasted value.</t>
         </is>
       </c>
       <c r="F7" s="5" t="inlineStr">
         <is>
-          <t>Copy action succeeds without errors.
-Clipboard contains a value matching the displayed parentUrn.</t>
+          <t>Pasted value matches the copied parentUrn exactly.
+No extra spaces, line breaks, or altered characters are introduced.</t>
         </is>
       </c>
       <c r="G7" s="5" t="inlineStr"/>
@@ -973,7 +973,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K5"/>
+  <dimension ref="A1:K6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -1188,7 +1188,7 @@
       </c>
       <c r="F4" s="5" t="inlineStr">
         <is>
-          <t>UAT-004, UAT-005</t>
+          <t>UAT-004</t>
         </is>
       </c>
       <c r="G4" s="5" t="inlineStr">
@@ -1271,6 +1271,63 @@
       <c r="K5" s="5" t="inlineStr">
         <is>
           <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="34" customHeight="1">
+      <c r="A6" s="5" t="inlineStr">
+        <is>
+          <t>COV-005</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="inlineStr">
+        <is>
+          <t>G2-20728</t>
+        </is>
+      </c>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>AC4</t>
+        </is>
+      </c>
+      <c r="D6" s="5" t="inlineStr">
+        <is>
+          <t>Copied parentUrn pastes into Concierge without formatting issues</t>
+        </is>
+      </c>
+      <c r="E6" s="5" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="F6" s="5" t="inlineStr">
+        <is>
+          <t>UAT-007</t>
+        </is>
+      </c>
+      <c r="G6" s="5" t="inlineStr">
+        <is>
+          <t>Full</t>
+        </is>
+      </c>
+      <c r="H6" s="5" t="inlineStr">
+        <is>
+          <t>Directly mapped to copy/paste outcome in Concierge</t>
+        </is>
+      </c>
+      <c r="I6" s="5" t="inlineStr">
+        <is>
+          <t>Unavailable</t>
+        </is>
+      </c>
+      <c r="J6" s="5" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="K6" s="5" t="inlineStr">
+        <is>
+          <t>No explicit constraints documented for allowed character formats in parentUrn</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: update UAT summary report formatting and improve dropped checks table
</commit_message>
<xml_diff>
--- a/uat-test-plans-reduced30/G2-16011-view-of-the-customer-customer-information.xlsx
+++ b/uat-test-plans-reduced30/G2-16011-view-of-the-customer-customer-information.xlsx
@@ -597,7 +597,7 @@
       </c>
       <c r="B12" s="3" t="inlineStr">
         <is>
-          <t>[Reduced V2 ~25% — 6/8 checks retained; AC and core-case coverage guardrails enforced] 1 UI story (G2-20728) mapped to 8 business checks and 5 AC coverage rows. 1 evaluation spike (G2-25652) excluded from executable UAT scope.</t>
+          <t>[Reduced V2 ~25% — 6/8 checks retained; AC coverage guardrail enforced] 1 UI story (G2-20728) mapped to 8 business checks and 5 AC coverage rows. 1 evaluation spike (G2-25652) excluded from executable UAT scope.</t>
         </is>
       </c>
     </row>
@@ -669,7 +669,7 @@
       </c>
       <c r="B18" s="3" t="inlineStr">
         <is>
-          <t>payload_bytes=7993; payload_chars=7979; est_tokens~1995; checklist_rows=6; matrix_rows=5; exploratory_rows=2</t>
+          <t>payload_bytes=7978; payload_chars=7964; est_tokens~1991; checklist_rows=6; matrix_rows=5; exploratory_rows=2</t>
         </is>
       </c>
     </row>

</xml_diff>